<commit_message>
Reserve TA cable space and fit KM05T ports on splitting board
</commit_message>
<xml_diff>
--- a/Production/TABoardV9/TA_Board_V9.xlsx
+++ b/Production/TABoardV9/TA_Board_V9.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R04db22a932494714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R73542c878b8f4a1b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>TA board V9.8 compact</x:v>
+        <x:v>TA board V9.9</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -396,7 +396,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>TA_Board_V9_baseplate_14x17p5in.step</x:v>
+        <x:v>TA_Board_V9_baseplate_14x21p5in.step</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
         <x:v>1</x:v>
@@ -696,7 +696,7 @@
     </x:row>
     <x:row r="54" ht="44" customHeight="1">
       <x:c r="A54" s="10" t="str">
-        <x:v>10. HKTS-5/64 adjusters are included with M05 / KA05T assemblies when purchased as kits; do not order them twice.</x:v>
+        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
       </x:c>
       <x:c r="B54" s="4"/>
     </x:row>

</xml_diff>

<commit_message>
Fold TA output across the board and shorten plate to 16.5 inches
</commit_message>
<xml_diff>
--- a/Production/TABoardV9/TA_Board_V9.xlsx
+++ b/Production/TABoardV9/TA_Board_V9.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R73542c878b8f4a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rd3273f4695924daa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>TA board V9.9</x:v>
+        <x:v>TA board V9.10</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -396,7 +396,7 @@
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>TA_Board_V9_baseplate_14x21p5in.step</x:v>
+        <x:v>TA_Board_V9_baseplate_14x16p5in.step</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
         <x:v>1</x:v>
@@ -435,7 +435,7 @@
         <x:v>1/2 in mirror (BB05-E03 or equivalent)</x:v>
       </x:c>
       <x:c r="B18" s="4" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -499,7 +499,7 @@
         <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
       </x:c>
       <x:c r="B26" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -555,7 +555,7 @@
         <x:v>Newport M05 mirror mount</x:v>
       </x:c>
       <x:c r="B33" s="4" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
@@ -654,7 +654,7 @@
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="2" t="str">
-        <x:v>3. Plate holes: 54 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
+        <x:v>3. Plate holes: 55 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
       </x:c>
       <x:c r="B47" s="4"/>
     </x:row>

</xml_diff>

<commit_message>
Compact TA to a single fiber output on a 14x11 inch table-grid plate
</commit_message>
<xml_diff>
--- a/Production/TABoardV9/TA_Board_V9.xlsx
+++ b/Production/TABoardV9/TA_Board_V9.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6d0e1e576858401e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re3ae6de33845438f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>TA board V9.11</x:v>
+        <x:v>TA board V9.12</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -324,15 +324,15 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="2" t="str">
-        <x:v>AOM_Adapter.step (upper adapter; lower seat is integral)</x:v>
+        <x:v>Rb_Cell_Enclosure_Cover_V9_7.step</x:v>
       </x:c>
       <x:c r="B4" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="2" t="str">
-        <x:v>Cube_Mount_Halfinch.step</x:v>
+        <x:v>Rb_Cell_Enclosure_Lid_V9_7.step</x:v>
       </x:c>
       <x:c r="B5" s="4" t="n">
         <x:v>1</x:v>
@@ -340,7 +340,7 @@
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="2" t="str">
-        <x:v>Iris_Mount.step (IDA12 slide mount)</x:v>
+        <x:v>Rb_Cell_Enclosure_LowerHalf_V9_7.step</x:v>
       </x:c>
       <x:c r="B6" s="4" t="n">
         <x:v>1</x:v>
@@ -348,23 +348,23 @@
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="2" t="str">
-        <x:v>Rb_Cell_Enclosure_Cover_V9_7.step</x:v>
+        <x:v>Surface_Adapter_isolator_lip.step</x:v>
       </x:c>
       <x:c r="B7" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="2" t="str">
-        <x:v>Rb_Cell_Enclosure_Lid_V9_7.step</x:v>
+        <x:v>Surface_Adapter_rsp05_lip.step</x:v>
       </x:c>
       <x:c r="B8" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>Rb_Cell_Enclosure_LowerHalf_V9_7.step</x:v>
+        <x:v>TA_Board_V9_baseplate_14x11in.step</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>1</x:v>
@@ -372,75 +372,75 @@
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="2" t="str">
-        <x:v>Shutter_Adapter.step</x:v>
+        <x:v>TA_adapter_board_model.step</x:v>
       </x:c>
       <x:c r="B10" s="4" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="2" t="str">
-        <x:v>Surface_Adapter_isolator_lip.step</x:v>
-      </x:c>
-      <x:c r="B11" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="A11" s="2"/>
+      <x:c r="B11" s="4"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="2" t="str">
-        <x:v>Surface_Adapter_rsp05_lip.step</x:v>
-      </x:c>
-      <x:c r="B12" s="4" t="n">
-        <x:v>7</x:v>
+      <x:c r="A12" s="8" t="str">
+        <x:v>Elements</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="str">
+        <x:v>#</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>TA_Board_V9_baseplate_14x16p5in.step</x:v>
+        <x:v>1/2 in half-wave (HWP) waveplate</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>TA_adapter.step</x:v>
+        <x:v>1/2 in mirror (BB05-E03 or equivalent)</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="2"/>
-      <x:c r="B15" s="4"/>
+      <x:c r="A15" s="2" t="str">
+        <x:v>1/2 in quarter-wave (QWP) waveplate</x:v>
+      </x:c>
+      <x:c r="B15" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="8" t="str">
-        <x:v>Elements</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="str">
-        <x:v>#</x:v>
+      <x:c r="A16" s="2" t="str">
+        <x:v>1/4-20 table bolt (baseplate fixing)</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>1/2 in half-wave (HWP) waveplate</x:v>
+        <x:v>8-32 x 2 in socket head screw (cell through-slot; not modelled)</x:v>
       </x:c>
       <x:c r="B17" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>1/2 in mirror (BB05-E03 or equivalent)</x:v>
+        <x:v>8-32 x 5/8 in socket head screw (cell end covers; not modelled)</x:v>
       </x:c>
       <x:c r="B18" s="4" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>1/2 in quarter-wave (QWP) waveplate</x:v>
+        <x:v>C220TMD-A fiber lens</x:v>
       </x:c>
       <x:c r="B19" s="4" t="n">
         <x:v>1</x:v>
@@ -448,39 +448,39 @@
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="2" t="str">
-        <x:v>1/4-20 table bolt (baseplate fixing)</x:v>
+        <x:v>GC25075-RB rubidium vapour cell (CAD envelope)</x:v>
       </x:c>
       <x:c r="B20" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="2" t="str">
-        <x:v>8-32 x 2 in socket head screw (cell through-slot; not modelled)</x:v>
+        <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
       </x:c>
       <x:c r="B21" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="2" t="str">
-        <x:v>8-32 x 5/8 in socket head screw (cell end covers; not modelled)</x:v>
+        <x:v>IOT-5-850-VLP isolator</x:v>
       </x:c>
       <x:c r="B22" s="4" t="n">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="2" t="str">
-        <x:v>C220TMD-A fiber lens</x:v>
+        <x:v>KA05T fiber port mount</x:v>
       </x:c>
       <x:c r="B23" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="2" t="str">
-        <x:v>G&amp;H AOMO 3100-125</x:v>
+        <x:v>Lens LA1289-B</x:v>
       </x:c>
       <x:c r="B24" s="4" t="n">
         <x:v>1</x:v>
@@ -488,7 +488,7 @@
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="2" t="str">
-        <x:v>GC25075-RB rubidium vapour cell (CAD envelope)</x:v>
+        <x:v>Lens LA1540-B</x:v>
       </x:c>
       <x:c r="B25" s="4" t="n">
         <x:v>1</x:v>
@@ -496,15 +496,15 @@
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2" t="str">
-        <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
+        <x:v>Newport M05 mirror mount</x:v>
       </x:c>
       <x:c r="B26" s="4" t="n">
-        <x:v>22</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="2" t="str">
-        <x:v>IDA12-P5 iris</x:v>
+        <x:v>PBS cube 12.7 mm</x:v>
       </x:c>
       <x:c r="B27" s="4" t="n">
         <x:v>1</x:v>
@@ -512,23 +512,23 @@
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="2" t="str">
-        <x:v>IOT-5-850-VLP isolator</x:v>
+        <x:v>POLARIS-L05G lens holder (no pin slots)</x:v>
       </x:c>
       <x:c r="B28" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="2" t="str">
-        <x:v>KA05T fiber port mount</x:v>
+        <x:v>RSP05 rotation mount</x:v>
       </x:c>
       <x:c r="B29" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="2" t="str">
-        <x:v>KM100PM (bridged)</x:v>
+        <x:v>S05TM09 lens adapter</x:v>
       </x:c>
       <x:c r="B30" s="4" t="n">
         <x:v>1</x:v>
@@ -536,169 +536,97 @@
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="2" t="str">
-        <x:v>Lens LA1289-B</x:v>
+        <x:v>SM05FCA2 fiber adapter</x:v>
       </x:c>
       <x:c r="B31" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="2" t="str">
-        <x:v>Lens LA1540-B</x:v>
+        <x:v>SM05L05 lens tube</x:v>
       </x:c>
       <x:c r="B32" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>Newport M05 mirror mount</x:v>
+        <x:v>TA butterfly package (TAboard), on TA adapter</x:v>
       </x:c>
       <x:c r="B33" s="4" t="n">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
-      <x:c r="A34" s="2" t="str">
-        <x:v>PBS cube 12.7 mm</x:v>
-      </x:c>
-      <x:c r="B34" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="A34" s="2"/>
+      <x:c r="B34" s="4"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
-      <x:c r="A35" s="2" t="str">
-        <x:v>PBS cube bonded to empty output RSP05 (not modelled)</x:v>
-      </x:c>
-      <x:c r="B35" s="4" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="24" customHeight="1">
-      <x:c r="A36" s="2" t="str">
-        <x:v>POLARIS-L05G lens holder (no pin slots)</x:v>
-      </x:c>
-      <x:c r="B36" s="4" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="24" customHeight="1">
-      <x:c r="A37" s="2" t="str">
-        <x:v>RSP05 rotation mount</x:v>
-      </x:c>
-      <x:c r="B37" s="4" t="n">
-        <x:v>7</x:v>
-      </x:c>
+      <x:c r="A35" s="8" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+      <x:c r="B35" s="9"/>
+    </x:row>
+    <x:row r="36" ht="44" customHeight="1">
+      <x:c r="A36" s="10" t="str">
+        <x:v>1. Modelled component quantities: TA_Board_V9_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+      </x:c>
+      <x:c r="B36" s="4"/>
+    </x:row>
+    <x:row r="37" ht="44" customHeight="1">
+      <x:c r="A37" s="10" t="str">
+        <x:v>2. Tapping classification: TA_Board_V9_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
+      </x:c>
+      <x:c r="B37" s="4"/>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="2" t="str">
-        <x:v>S05TM09 lens adapter</x:v>
-      </x:c>
-      <x:c r="B38" s="4" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="24" customHeight="1">
-      <x:c r="A39" s="2" t="str">
-        <x:v>SM05FCA2 fiber adapter</x:v>
-      </x:c>
-      <x:c r="B39" s="4" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="24" customHeight="1">
-      <x:c r="A40" s="2" t="str">
-        <x:v>SM05L05 lens tube</x:v>
-      </x:c>
-      <x:c r="B40" s="4" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="24" customHeight="1">
-      <x:c r="A41" s="2" t="str">
-        <x:v>SRS SR475 shutter</x:v>
-      </x:c>
-      <x:c r="B41" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="24" customHeight="1">
-      <x:c r="A42" s="2" t="str">
-        <x:v>TA butterfly package (TAboard), on TA adapter</x:v>
-      </x:c>
-      <x:c r="B42" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="24" customHeight="1">
-      <x:c r="A43" s="2"/>
+        <x:v>3. Plate holes: 33 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
+      </x:c>
+      <x:c r="B38" s="4"/>
+    </x:row>
+    <x:row r="39" ht="44" customHeight="1">
+      <x:c r="A39" s="10" t="str">
+        <x:v>4. The TA butterfly package mounts to the TA adapter. Its small adapter threads are not baseplate taps.</x:v>
+      </x:c>
+      <x:c r="B39" s="4"/>
+    </x:row>
+    <x:row r="40" ht="44" customHeight="1">
+      <x:c r="A40" s="10" t="str">
+        <x:v>5. 6 bare conditioning stations are drilled provisions. No holder or optic is installed there.</x:v>
+      </x:c>
+      <x:c r="B40" s="4"/>
+    </x:row>
+    <x:row r="41" ht="62" customHeight="1">
+      <x:c r="A41" s="10" t="str">
+        <x:v>6. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+      </x:c>
+      <x:c r="B41" s="4"/>
+    </x:row>
+    <x:row r="42" ht="62" customHeight="1">
+      <x:c r="A42" s="10" t="str">
+        <x:v>7. The TA has one direct fiber output after the rubidium cell: mirror, first lens, mirror, second lens, HWP, bonded rotating PBS and KA05T fiber port. The folded distance between the two lenses is 45.319348 mm.</x:v>
+      </x:c>
+      <x:c r="B42" s="4"/>
+    </x:row>
+    <x:row r="43" ht="44" customHeight="1">
+      <x:c r="A43" s="10" t="str">
+        <x:v>8. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
+      </x:c>
       <x:c r="B43" s="4"/>
     </x:row>
-    <x:row r="44" ht="24" customHeight="1">
-      <x:c r="A44" s="8" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="B44" s="9"/>
+    <x:row r="44" ht="44" customHeight="1">
+      <x:c r="A44" s="10" t="str">
+        <x:v>9. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
+      </x:c>
+      <x:c r="B44" s="4"/>
     </x:row>
     <x:row r="45" ht="44" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>1. Modelled component quantities: TA_Board_V9_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
       </x:c>
       <x:c r="B45" s="4"/>
-    </x:row>
-    <x:row r="46" ht="44" customHeight="1">
-      <x:c r="A46" s="10" t="str">
-        <x:v>2. Tapping classification: TA_Board_V9_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
-      </x:c>
-      <x:c r="B46" s="4"/>
-    </x:row>
-    <x:row r="47" ht="24" customHeight="1">
-      <x:c r="A47" s="2" t="str">
-        <x:v>3. Plate holes: 55 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
-      </x:c>
-      <x:c r="B47" s="4"/>
-    </x:row>
-    <x:row r="48" ht="44" customHeight="1">
-      <x:c r="A48" s="10" t="str">
-        <x:v>4. AOM lower seats are integral with the baseplate. Only the upper AOM adapter is a separate part.</x:v>
-      </x:c>
-      <x:c r="B48" s="4"/>
-    </x:row>
-    <x:row r="49" ht="44" customHeight="1">
-      <x:c r="A49" s="10" t="str">
-        <x:v>5. The TA butterfly package mounts to the TA adapter. Its small adapter threads are not baseplate taps.</x:v>
-      </x:c>
-      <x:c r="B49" s="4"/>
-    </x:row>
-    <x:row r="50" ht="44" customHeight="1">
-      <x:c r="A50" s="10" t="str">
-        <x:v>6. 6 bare conditioning stations are drilled provisions. No holder or optic is installed there.</x:v>
-      </x:c>
-      <x:c r="B50" s="4"/>
-    </x:row>
-    <x:row r="51" ht="44" customHeight="1">
-      <x:c r="A51" s="10" t="str">
-        <x:v>7. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
-      </x:c>
-      <x:c r="B51" s="4"/>
-    </x:row>
-    <x:row r="52" ht="44" customHeight="1">
-      <x:c r="A52" s="10" t="str">
-        <x:v>8. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
-      </x:c>
-      <x:c r="B52" s="4"/>
-    </x:row>
-    <x:row r="53" ht="44" customHeight="1">
-      <x:c r="A53" s="10" t="str">
-        <x:v>9. The 2 empty output RSP05 mounts each require one bonded PBS cube, listed separately because it is not modelled.</x:v>
-      </x:c>
-      <x:c r="B53" s="4"/>
-    </x:row>
-    <x:row r="54" ht="44" customHeight="1">
-      <x:c r="A54" s="10" t="str">
-        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
-      </x:c>
-      <x:c r="B54" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Compact TA V9.13 to 11.625 by 11 inches with four lens provisions
</commit_message>
<xml_diff>
--- a/Production/TABoardV9/TA_Board_V9.xlsx
+++ b/Production/TABoardV9/TA_Board_V9.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re3ae6de33845438f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5cc0c6f4ecb843ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>TA board V9.12</x:v>
+        <x:v>TA board V9.13</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -364,7 +364,7 @@
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>TA_Board_V9_baseplate_14x11in.step</x:v>
+        <x:v>TA_Board_V9_baseplate_11p625x11in.step</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>1</x:v>
@@ -582,7 +582,7 @@
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="2" t="str">
-        <x:v>3. Plate holes: 33 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
+        <x:v>3. Plate holes: 31 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
       </x:c>
       <x:c r="B38" s="4"/>
     </x:row>
@@ -594,7 +594,7 @@
     </x:row>
     <x:row r="40" ht="44" customHeight="1">
       <x:c r="A40" s="10" t="str">
-        <x:v>5. 6 bare conditioning stations are drilled provisions. No holder or optic is installed there.</x:v>
+        <x:v>5. 4 bare conditioning stations provide 2 cylindrical-lens and 2 spherical-lens mounting positions. Holders and optics remain unselected and are not installed or counted in this BOM.</x:v>
       </x:c>
       <x:c r="B40" s="4"/>
     </x:row>
@@ -610,23 +610,29 @@
       </x:c>
       <x:c r="B42" s="4"/>
     </x:row>
-    <x:row r="43" ht="44" customHeight="1">
+    <x:row r="43" ht="62" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>8. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
+        <x:v>8. The upstream HWP is on the first horizontal TA output leg, before the first steering mirror. The QWP is on the left vertical leg, after the isolator and before the conditioning stations.</x:v>
       </x:c>
       <x:c r="B43" s="4"/>
     </x:row>
     <x:row r="44" ht="44" customHeight="1">
       <x:c r="A44" s="10" t="str">
-        <x:v>9. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
+        <x:v>9. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
       </x:c>
       <x:c r="B44" s="4"/>
     </x:row>
     <x:row r="45" ht="44" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+        <x:v>10. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
       </x:c>
       <x:c r="B45" s="4"/>
+    </x:row>
+    <x:row r="46" ht="44" customHeight="1">
+      <x:c r="A46" s="10" t="str">
+        <x:v>11. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+      </x:c>
+      <x:c r="B46" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Trim TA board and restore upstream waveplate order with verified L05G fit
</commit_message>
<xml_diff>
--- a/Production/TABoardV9/TA_Board_V9.xlsx
+++ b/Production/TABoardV9/TA_Board_V9.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5cc0c6f4ecb843ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7f9b242bdd534a22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>TA board V9.13</x:v>
+        <x:v>TA board V9.14 - 11.625 x 10.15 in</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -364,7 +364,7 @@
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="2" t="str">
-        <x:v>TA_Board_V9_baseplate_11p625x11in.step</x:v>
+        <x:v>TA_Board_V9_baseplate_11p625x10p15in.step</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
         <x:v>1</x:v>
@@ -512,31 +512,31 @@
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="2" t="str">
-        <x:v>POLARIS-L05G lens holder (no pin slots)</x:v>
+        <x:v>POLARIS-L05G lens holder (four planned conditioning positions)</x:v>
       </x:c>
       <x:c r="B28" s="4" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="2" t="str">
-        <x:v>RSP05 rotation mount</x:v>
+        <x:v>POLARIS-L05G lens holder (no pin slots)</x:v>
       </x:c>
       <x:c r="B29" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="2" t="str">
-        <x:v>S05TM09 lens adapter</x:v>
+        <x:v>RSP05 rotation mount</x:v>
       </x:c>
       <x:c r="B30" s="4" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="2" t="str">
-        <x:v>SM05FCA2 fiber adapter</x:v>
+        <x:v>S05TM09 lens adapter</x:v>
       </x:c>
       <x:c r="B31" s="4" t="n">
         <x:v>1</x:v>
@@ -544,7 +544,7 @@
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="2" t="str">
-        <x:v>SM05L05 lens tube</x:v>
+        <x:v>SM05FCA2 fiber adapter</x:v>
       </x:c>
       <x:c r="B32" s="4" t="n">
         <x:v>1</x:v>
@@ -552,87 +552,95 @@
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="2" t="str">
+        <x:v>SM05L05 lens tube</x:v>
+      </x:c>
+      <x:c r="B33" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="24" customHeight="1">
+      <x:c r="A34" s="2" t="str">
         <x:v>TA butterfly package (TAboard), on TA adapter</x:v>
       </x:c>
-      <x:c r="B33" s="4" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="24" customHeight="1">
-      <x:c r="A34" s="2"/>
-      <x:c r="B34" s="4"/>
+      <x:c r="B34" s="4" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
-      <x:c r="A35" s="8" t="str">
+      <x:c r="A35" s="2"/>
+      <x:c r="B35" s="4"/>
+    </x:row>
+    <x:row r="36" ht="24" customHeight="1">
+      <x:c r="A36" s="8" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="B35" s="9"/>
-    </x:row>
-    <x:row r="36" ht="44" customHeight="1">
-      <x:c r="A36" s="10" t="str">
-        <x:v>1. Modelled component quantities: TA_Board_V9_validation.json. Adapter filenames follow Production/Adapters.</x:v>
-      </x:c>
-      <x:c r="B36" s="4"/>
+      <x:c r="B36" s="9"/>
     </x:row>
     <x:row r="37" ht="44" customHeight="1">
       <x:c r="A37" s="10" t="str">
+        <x:v>1. Modelled component quantities: TA_Board_V9_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+      </x:c>
+      <x:c r="B37" s="4"/>
+    </x:row>
+    <x:row r="38" ht="44" customHeight="1">
+      <x:c r="A38" s="10" t="str">
         <x:v>2. Tapping classification: TA_Board_V9_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
       </x:c>
-      <x:c r="B37" s="4"/>
-    </x:row>
-    <x:row r="38" ht="24" customHeight="1">
-      <x:c r="A38" s="2" t="str">
+      <x:c r="B38" s="4"/>
+    </x:row>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="2" t="str">
         <x:v>3. Plate holes: 31 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
-      </x:c>
-      <x:c r="B38" s="4"/>
-    </x:row>
-    <x:row r="39" ht="44" customHeight="1">
-      <x:c r="A39" s="10" t="str">
-        <x:v>4. The TA butterfly package mounts to the TA adapter. Its small adapter threads are not baseplate taps.</x:v>
       </x:c>
       <x:c r="B39" s="4"/>
     </x:row>
     <x:row r="40" ht="44" customHeight="1">
       <x:c r="A40" s="10" t="str">
-        <x:v>5. 4 bare conditioning stations provide 2 cylindrical-lens and 2 spherical-lens mounting positions. Holders and optics remain unselected and are not installed or counted in this BOM.</x:v>
+        <x:v>4. The TA butterfly package mounts to the TA adapter. Its small adapter threads are not baseplate taps.</x:v>
       </x:c>
       <x:c r="B40" s="4"/>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
       <x:c r="A41" s="10" t="str">
-        <x:v>6. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+        <x:v>5. 4 bare conditioning stations provide 2 cylindrical-lens and 2 spherical-lens positions. Four selected POLARIS-L05G holders are listed as planned parts; actual native holder/cutter fit is verified, while optics remain unselected.</x:v>
       </x:c>
       <x:c r="B41" s="4"/>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
       <x:c r="A42" s="10" t="str">
-        <x:v>7. The TA has one direct fiber output after the rubidium cell: mirror, first lens, mirror, second lens, HWP, bonded rotating PBS and KA05T fiber port. The folded distance between the two lenses is 45.319348 mm.</x:v>
+        <x:v>6. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
       </x:c>
       <x:c r="B42" s="4"/>
     </x:row>
     <x:row r="43" ht="62" customHeight="1">
       <x:c r="A43" s="10" t="str">
-        <x:v>8. The upstream HWP is on the first horizontal TA output leg, before the first steering mirror. The QWP is on the left vertical leg, after the isolator and before the conditioning stations.</x:v>
+        <x:v>7. The TA has one direct fiber output after the rubidium cell: mirror, first lens, mirror, second lens, HWP, bonded rotating PBS and KA05T fiber port. The folded distance between the two lenses is 45.319348 mm.</x:v>
       </x:c>
       <x:c r="B43" s="4"/>
     </x:row>
-    <x:row r="44" ht="44" customHeight="1">
+    <x:row r="44" ht="62" customHeight="1">
       <x:c r="A44" s="10" t="str">
-        <x:v>9. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
+        <x:v>8. Original upstream order restored: TA -&gt; two steering mirrors -&gt; HWP -&gt; isolator -&gt; QWP -&gt; common folding mirrors and conditioning. Actual native optical centres, axes and mirror normals are independently checked.</x:v>
       </x:c>
       <x:c r="B44" s="4"/>
     </x:row>
     <x:row r="45" ht="44" customHeight="1">
       <x:c r="A45" s="10" t="str">
-        <x:v>10. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
+        <x:v>9. The V9.7 cell lower half, lid and covers reuse the STEP files in Production/CellEnclosure. The seat pocket and mounting taps are baseplate machining, not separate parts.</x:v>
       </x:c>
       <x:c r="B45" s="4"/>
     </x:row>
     <x:row r="46" ht="44" customHeight="1">
       <x:c r="A46" s="10" t="str">
+        <x:v>10. The supplied V9.7 front and rear cell covers are opaque and have no beam apertures. Machine the beam apertures before optical operation; their present geometry blocks the beam.</x:v>
+      </x:c>
+      <x:c r="B46" s="4"/>
+    </x:row>
+    <x:row r="47" ht="44" customHeight="1">
+      <x:c r="A47" s="10" t="str">
         <x:v>11. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
       </x:c>
-      <x:c r="B46" s="4"/>
+      <x:c r="B47" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>